<commit_message>
CRUD minus Delete operation in comment and post
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Coding\WD\NE\backend\03_yt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69CEE2C6-894D-4729-88B3-BFDF53A406EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5432DA45-BFAA-491C-9BBE-647C6DF40F5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{334C76F3-0857-41C1-B9BD-0792E94EC8EC}"/>
+    <workbookView xWindow="492" yWindow="2712" windowWidth="11064" windowHeight="9120" xr2:uid="{334C76F3-0857-41C1-B9BD-0792E94EC8EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -84,12 +84,6 @@
     <t>Mohit Ranjan</t>
   </si>
   <si>
-    <t>mohitranjan2111@gmail.com</t>
-  </si>
-  <si>
-    <t>greatBrother@1</t>
-  </si>
-  <si>
     <t>user 3</t>
   </si>
   <si>
@@ -124,6 +118,12 @@
   </si>
   <si>
     <t>testy21@gmail.com</t>
+  </si>
+  <si>
+    <t>mohitr2111@gmail.com</t>
+  </si>
+  <si>
+    <t>MOHO</t>
   </si>
 </sst>
 </file>
@@ -179,10 +179,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -503,209 +503,209 @@
   <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.6640625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="27.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="2"/>
-    <col min="4" max="5" width="16.88671875" style="2" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="11.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" style="1"/>
+    <col min="4" max="5" width="16.88671875" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="D1" s="1" t="s">
+      <c r="B1" s="3"/>
+      <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="D7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="3"/>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="D7" s="1" t="s">
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="D13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E13" s="3"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
+      <c r="D16" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E10" s="2" t="s">
+      <c r="E16" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+      <c r="D17" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="1"/>
-      <c r="D13" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E13" s="1"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>22</v>
+      <c r="E17" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -722,6 +722,7 @@
     <hyperlink ref="B5" r:id="rId1" xr:uid="{45953EBB-8E0B-4D83-93A6-84074A20F7F3}"/>
     <hyperlink ref="B15" r:id="rId2" xr:uid="{9DAE5C10-D9D3-4728-9FD9-CAEDE5DFC7B1}"/>
     <hyperlink ref="E15" r:id="rId3" xr:uid="{E7EC750C-4EA9-4D77-8DE8-1FA98FC957D1}"/>
+    <hyperlink ref="B9" r:id="rId4" xr:uid="{2269E30E-FA4B-47BE-A159-177787431777}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
complete aggregation #1 user profile endpoint and full backend testing
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Coding\WD\NE\backend\03_yt\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5432DA45-BFAA-491C-9BBE-647C6DF40F5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90954DE0-5917-4BA8-B898-1E0DCD3186B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="492" yWindow="2712" windowWidth="11064" windowHeight="9120" xr2:uid="{334C76F3-0857-41C1-B9BD-0792E94EC8EC}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{334C76F3-0857-41C1-B9BD-0792E94EC8EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="84">
   <si>
     <t>user 1</t>
   </si>
@@ -123,14 +123,176 @@
     <t>mohitr2111@gmail.com</t>
   </si>
   <si>
-    <t>MOHO</t>
+    <t>user 5</t>
+  </si>
+  <si>
+    <t>user 6</t>
+  </si>
+  <si>
+    <t>Checklist</t>
+  </si>
+  <si>
+    <t>register User</t>
+  </si>
+  <si>
+    <t>login user</t>
+  </si>
+  <si>
+    <t>logout user</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Reset Refresh token</t>
+  </si>
+  <si>
+    <t>change password</t>
+  </si>
+  <si>
+    <t>curr user</t>
+  </si>
+  <si>
+    <t>update fullname</t>
+  </si>
+  <si>
+    <t>update email</t>
+  </si>
+  <si>
+    <t>update avatar</t>
+  </si>
+  <si>
+    <t>update coverImage</t>
+  </si>
+  <si>
+    <t>get user profile</t>
+  </si>
+  <si>
+    <t>get watch history</t>
+  </si>
+  <si>
+    <t>delete user</t>
+  </si>
+  <si>
+    <t>MOH1</t>
+  </si>
+  <si>
+    <t>USER</t>
+  </si>
+  <si>
+    <t>upload video</t>
+  </si>
+  <si>
+    <t>update video details</t>
+  </si>
+  <si>
+    <t>change thumbnail</t>
+  </si>
+  <si>
+    <t>watch video</t>
+  </si>
+  <si>
+    <t>list unlist video</t>
+  </si>
+  <si>
+    <t>delete video</t>
+  </si>
+  <si>
+    <t>VIDEO</t>
+  </si>
+  <si>
+    <t>create post</t>
+  </si>
+  <si>
+    <t>get post</t>
+  </si>
+  <si>
+    <t>update post</t>
+  </si>
+  <si>
+    <t>POST</t>
+  </si>
+  <si>
+    <t>on video</t>
+  </si>
+  <si>
+    <t>on post</t>
+  </si>
+  <si>
+    <t>on playlist</t>
+  </si>
+  <si>
+    <t>on comment</t>
+  </si>
+  <si>
+    <t>get video rxn</t>
+  </si>
+  <si>
+    <t>get post rxn</t>
+  </si>
+  <si>
+    <t>get playlist rxn</t>
+  </si>
+  <si>
+    <t>get comment rxn</t>
+  </si>
+  <si>
+    <t>LIKE</t>
+  </si>
+  <si>
+    <t>on reply</t>
+  </si>
+  <si>
+    <t>update comment</t>
+  </si>
+  <si>
+    <t>get comment reply</t>
+  </si>
+  <si>
+    <t>COMMENT</t>
+  </si>
+  <si>
+    <t>create playlist</t>
+  </si>
+  <si>
+    <t>get playlist</t>
+  </si>
+  <si>
+    <t>upadte playlist</t>
+  </si>
+  <si>
+    <t>add video to playlist</t>
+  </si>
+  <si>
+    <t>get users playlist</t>
+  </si>
+  <si>
+    <t>PLAYLIST</t>
+  </si>
+  <si>
+    <t>subscribe channel</t>
+  </si>
+  <si>
+    <t>subscribers details</t>
+  </si>
+  <si>
+    <t>subscribed channels</t>
+  </si>
+  <si>
+    <t>SUBSCRIPTION</t>
+  </si>
+  <si>
+    <t>subscription status</t>
+  </si>
+  <si>
+    <t>special case of array</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -152,18 +314,255 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="36"/>
+      <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="28"/>
+      <color theme="2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="13">
     <border>
       <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color theme="2"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="2"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color theme="2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color theme="2"/>
+      </right>
+      <top style="medium">
+        <color theme="2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="2"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="2"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top style="medium">
+        <color theme="2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top style="medium">
+        <color theme="2"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="medium">
+        <color theme="2"/>
+      </right>
+      <top style="medium">
+        <color theme="2"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
+      <right style="thin">
+        <color theme="2"/>
+      </right>
+      <top style="thin">
+        <color theme="2"/>
+      </top>
+      <bottom style="medium">
+        <color theme="2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="2"/>
+      </left>
       <right/>
       <top/>
       <bottom/>
@@ -174,15 +573,117 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -500,216 +1001,634 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6428F8C0-E863-4A42-8004-C2F0813C83A1}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="27.6640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="8.88671875" style="1"/>
-    <col min="4" max="5" width="16.88671875" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="1"/>
+    <col min="4" max="6" width="16.88671875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.77734375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="18.44140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="15.88671875" style="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:9" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="D1" s="3" t="s">
+      <c r="B1" s="15"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="3"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="E1" s="15"/>
+      <c r="H1" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="C2" s="2"/>
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="G2" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" s="6"/>
+    </row>
+    <row r="3" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="C3" s="2"/>
+      <c r="D3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="G3" s="17"/>
+      <c r="H3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I3" s="6"/>
+    </row>
+    <row r="4" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="C4" s="2"/>
+      <c r="D4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
+      <c r="G4" s="17"/>
+      <c r="H4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="C5" s="2"/>
+      <c r="D5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+      <c r="F5" s="5"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I5" s="6"/>
+    </row>
+    <row r="6" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I6" s="6"/>
+    </row>
+    <row r="7" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="D7" s="3" t="s">
+      <c r="B7" s="15"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="3"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
+      <c r="E7" s="15"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" s="6"/>
+    </row>
+    <row r="8" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="C8" s="2"/>
+      <c r="D8" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
+      <c r="G8" s="17"/>
+      <c r="H8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="C9" s="2"/>
+      <c r="D9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="3" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+      <c r="F9" s="5"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I9" s="6"/>
+    </row>
+    <row r="10" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="C10" s="2"/>
+      <c r="D10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="G10" s="17"/>
+      <c r="H10" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I10" s="6"/>
+    </row>
+    <row r="11" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="5"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I11" s="6"/>
+    </row>
+    <row r="12" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="I12" s="8"/>
+    </row>
+    <row r="13" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="B13" s="15"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="15"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I13" s="6"/>
+    </row>
+    <row r="14" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" s="18"/>
+      <c r="H14" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I14" s="8"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="22"/>
+    </row>
+    <row r="16" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="22"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="3"/>
-      <c r="D13" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E13" s="3"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
+      <c r="C17" s="2"/>
+      <c r="D17" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="E17" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>20</v>
-      </c>
+      <c r="F17" s="5"/>
+      <c r="G17" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I17" s="7"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G18" s="20"/>
+      <c r="H18" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="I18" s="7"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G19" s="20"/>
+      <c r="H19" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="I19" s="7"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G20" s="20"/>
+      <c r="H20" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I20" s="7"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G21" s="20"/>
+      <c r="H21" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="I21" s="7"/>
+    </row>
+    <row r="22" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G22" s="21"/>
+      <c r="H22" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="I22" s="9"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
+      <c r="I23" s="22"/>
+    </row>
+    <row r="24" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+      <c r="I24" s="22"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G25" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I25" s="7"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G26" s="24"/>
+      <c r="H26" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="I26" s="7"/>
+    </row>
+    <row r="27" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G27" s="25"/>
+      <c r="H27" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="I27" s="7"/>
+      <c r="J27" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="K27" s="13"/>
+      <c r="L27" s="13"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="I28" s="22"/>
+    </row>
+    <row r="29" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
+      <c r="I29" s="22"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G30" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I30" s="7"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G31" s="33"/>
+      <c r="H31" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I31" s="7"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="G32" s="33"/>
+      <c r="H32" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I32" s="7"/>
+    </row>
+    <row r="33" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G33" s="33"/>
+      <c r="H33" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I33" s="7"/>
+    </row>
+    <row r="34" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G34" s="33"/>
+      <c r="H34" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I34" s="7"/>
+    </row>
+    <row r="35" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G35" s="33"/>
+      <c r="H35" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="I35" s="7"/>
+    </row>
+    <row r="36" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G36" s="33"/>
+      <c r="H36" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="I36" s="7"/>
+    </row>
+    <row r="37" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G37" s="34"/>
+      <c r="H37" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="I37" s="7"/>
+    </row>
+    <row r="38" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G38" s="22"/>
+      <c r="H38" s="22"/>
+      <c r="I38" s="22"/>
+    </row>
+    <row r="39" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G39" s="22"/>
+      <c r="H39" s="22"/>
+      <c r="I39" s="22"/>
+    </row>
+    <row r="40" spans="7:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G40" s="35" t="s">
+        <v>71</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="I40" s="7"/>
+    </row>
+    <row r="41" spans="7:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G41" s="36"/>
+      <c r="H41" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="I41" s="7"/>
+    </row>
+    <row r="42" spans="7:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G42" s="36"/>
+      <c r="H42" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="I42" s="7"/>
+    </row>
+    <row r="43" spans="7:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G43" s="36"/>
+      <c r="H43" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="I43" s="7"/>
+    </row>
+    <row r="44" spans="7:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G44" s="36"/>
+      <c r="H44" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I44" s="7"/>
+    </row>
+    <row r="45" spans="7:9" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G45" s="37"/>
+      <c r="H45" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I45" s="7"/>
+    </row>
+    <row r="46" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G46" s="22"/>
+      <c r="H46" s="22"/>
+      <c r="I46" s="22"/>
+    </row>
+    <row r="47" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G47" s="22"/>
+      <c r="H47" s="22"/>
+      <c r="I47" s="22"/>
+    </row>
+    <row r="48" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G48" s="26" t="s">
+        <v>77</v>
+      </c>
+      <c r="H48" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="I48" s="14"/>
+    </row>
+    <row r="49" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G49" s="27"/>
+      <c r="H49" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="I49" s="14"/>
+    </row>
+    <row r="50" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G50" s="27"/>
+      <c r="H50" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I50" s="14"/>
+    </row>
+    <row r="51" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G51" s="27"/>
+      <c r="H51" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="I51" s="14"/>
+    </row>
+    <row r="52" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G52" s="28"/>
+      <c r="H52" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="I52" s="14"/>
+    </row>
+    <row r="53" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G53" s="22"/>
+      <c r="H53" s="22"/>
+      <c r="I53" s="22"/>
+    </row>
+    <row r="54" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G54" s="22"/>
+      <c r="H54" s="22"/>
+      <c r="I54" s="22"/>
+    </row>
+    <row r="55" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G55" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="I55" s="7"/>
+    </row>
+    <row r="56" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G56" s="30"/>
+      <c r="H56" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="I56" s="7"/>
+    </row>
+    <row r="57" spans="7:9" x14ac:dyDescent="0.3">
+      <c r="G57" s="30"/>
+      <c r="H57" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I57" s="7"/>
+    </row>
+    <row r="58" spans="7:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="G58" s="31"/>
+      <c r="H58" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="I58" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="19">
+    <mergeCell ref="G48:G52"/>
+    <mergeCell ref="G53:I54"/>
+    <mergeCell ref="G55:G58"/>
+    <mergeCell ref="G30:G37"/>
+    <mergeCell ref="G28:I29"/>
+    <mergeCell ref="G38:I39"/>
+    <mergeCell ref="G40:G45"/>
+    <mergeCell ref="G46:I47"/>
+    <mergeCell ref="G2:G14"/>
+    <mergeCell ref="G17:G22"/>
+    <mergeCell ref="G15:I16"/>
+    <mergeCell ref="G23:I24"/>
+    <mergeCell ref="G25:G27"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="D1:E1"/>
     <mergeCell ref="A7:B7"/>
@@ -725,5 +1644,6 @@
     <hyperlink ref="B9" r:id="rId4" xr:uid="{2269E30E-FA4B-47BE-A159-177787431777}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>